<commit_message>
Updated confidence thresholds in species summary, and updated data cleaning to include all meta data, and additional control variable (deployment_ID).
</commit_message>
<xml_diff>
--- a/phase1_analysis/data/BD2025_species_summary.xlsx
+++ b/phase1_analysis/data/BD2025_species_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\Documents\University\Year 5 Masters\Research Project\2. Analysis\final_research_project\phase1_analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3B1C73-4B7E-4A05-9E69-E0B474217225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E9C9DB-0F53-4017-9F86-BBFC6D022BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -880,7 +880,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -891,7 +891,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3509,16 +3508,16 @@
       <c r="G67">
         <v>3</v>
       </c>
-      <c r="H67" s="6">
+      <c r="H67">
         <v>0.32</v>
       </c>
-      <c r="I67" s="6">
+      <c r="I67">
         <v>0.38</v>
       </c>
-      <c r="J67" s="6">
+      <c r="J67">
         <v>0.47</v>
       </c>
-      <c r="K67" s="6">
+      <c r="K67">
         <v>0.68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated species list, and wrote code to filter dataset by species-specific confidence thresholds. Will need to re-run if we manage to sort the last two species out, if not leave as is.
</commit_message>
<xml_diff>
--- a/phase1_analysis/data/BD2025_species_summary.xlsx
+++ b/phase1_analysis/data/BD2025_species_summary.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\Documents\University\Year 5 Masters\Research Project\2. Analysis\final_research_project\phase1_analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E9C9DB-0F53-4017-9F86-BBFC6D022BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B2EB98-D4A0-4FD1-82CE-792852E2DF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="269">
   <si>
     <t>common_n</t>
   </si>
@@ -818,6 +831,15 @@
   </si>
   <si>
     <t>false_pos</t>
+  </si>
+  <si>
+    <t>negative_corr</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>T</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K128"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.21875" bestFit="1" customWidth="1"/>
@@ -1205,9 +1227,10 @@
     <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="9.33203125" customWidth="1"/>
     <col min="8" max="11" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1241,8 +1264,11 @@
       <c r="K1" s="1" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1276,8 +1302,11 @@
       <c r="K2" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1311,8 +1340,11 @@
       <c r="K3">
         <v>0.59</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1346,8 +1378,11 @@
       <c r="K4" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L4" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1381,8 +1416,11 @@
       <c r="K5">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L5" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1416,8 +1454,11 @@
       <c r="K6" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1451,8 +1492,11 @@
       <c r="K7" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1486,8 +1530,11 @@
       <c r="K8" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L8" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1521,8 +1568,11 @@
       <c r="K9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L9" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1556,8 +1606,11 @@
       <c r="K10" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L10" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1591,8 +1644,11 @@
       <c r="K11" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L11" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1626,8 +1682,11 @@
       <c r="K12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L12" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -1658,8 +1717,11 @@
       <c r="J13">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L13" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -1693,8 +1755,11 @@
       <c r="K14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L14" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -1728,8 +1793,11 @@
       <c r="K15" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L15" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -1763,8 +1831,11 @@
       <c r="K16" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L16" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1798,8 +1869,11 @@
       <c r="K17" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L17" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -1833,8 +1907,11 @@
       <c r="K18">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L18" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -1868,8 +1945,11 @@
       <c r="K19" s="5" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L19" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -1903,8 +1983,11 @@
       <c r="K20" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L20" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -1938,8 +2021,11 @@
       <c r="K21" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L21" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>45</v>
       </c>
@@ -1973,8 +2059,11 @@
       <c r="K22" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L22" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>47</v>
       </c>
@@ -1990,12 +2079,29 @@
       <c r="E23">
         <v>0.95009999999999994</v>
       </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F23">
+        <v>87</v>
+      </c>
+      <c r="G23">
+        <v>13</v>
+      </c>
+      <c r="H23">
+        <v>0.35</v>
+      </c>
+      <c r="I23">
+        <v>0.42</v>
+      </c>
+      <c r="J23">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="K23">
+        <v>0.82</v>
+      </c>
+      <c r="L23" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>49</v>
       </c>
@@ -2011,12 +2117,29 @@
       <c r="E24">
         <v>0.82509999999999994</v>
       </c>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F24">
+        <v>28</v>
+      </c>
+      <c r="G24">
+        <v>72</v>
+      </c>
+      <c r="H24">
+        <v>0.85</v>
+      </c>
+      <c r="I24">
+        <v>0.94</v>
+      </c>
+      <c r="J24" t="s">
+        <v>263</v>
+      </c>
+      <c r="K24" t="s">
+        <v>263</v>
+      </c>
+      <c r="L24" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>51</v>
       </c>
@@ -2050,8 +2173,11 @@
       <c r="K25">
         <v>0.68</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L25" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -2085,8 +2211,11 @@
       <c r="K26">
         <v>0.87</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L26" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>55</v>
       </c>
@@ -2120,8 +2249,11 @@
       <c r="K27" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L27" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>57</v>
       </c>
@@ -2155,8 +2287,11 @@
       <c r="K28" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L28" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -2190,8 +2325,11 @@
       <c r="K29" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L29" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>61</v>
       </c>
@@ -2225,8 +2363,11 @@
       <c r="K30" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L30" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>63</v>
       </c>
@@ -2260,8 +2401,11 @@
       <c r="K31" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L31" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -2295,8 +2439,11 @@
       <c r="K32" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L32" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>67</v>
       </c>
@@ -2330,8 +2477,11 @@
       <c r="K33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L33" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -2365,8 +2515,11 @@
       <c r="K34" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L34" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>71</v>
       </c>
@@ -2400,8 +2553,11 @@
       <c r="K35">
         <v>0.72</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L35" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -2435,8 +2591,11 @@
       <c r="K36" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L36" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -2470,8 +2629,11 @@
       <c r="K37" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L37" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>77</v>
       </c>
@@ -2505,8 +2667,11 @@
       <c r="K38" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L38" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>79</v>
       </c>
@@ -2540,8 +2705,11 @@
       <c r="K39" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L39" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>81</v>
       </c>
@@ -2575,8 +2743,11 @@
       <c r="K40" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L40" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>83</v>
       </c>
@@ -2610,8 +2781,11 @@
       <c r="K41" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L41" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>85</v>
       </c>
@@ -2645,8 +2819,11 @@
       <c r="K42" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L42" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>87</v>
       </c>
@@ -2680,8 +2857,11 @@
       <c r="K43" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L43" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>89</v>
       </c>
@@ -2715,8 +2895,11 @@
       <c r="K44" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L44" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>91</v>
       </c>
@@ -2750,8 +2933,11 @@
       <c r="K45">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L45" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>93</v>
       </c>
@@ -2785,8 +2971,11 @@
       <c r="K46" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L46" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>95</v>
       </c>
@@ -2820,8 +3009,11 @@
       <c r="K47" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L47" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>97</v>
       </c>
@@ -2855,8 +3047,11 @@
       <c r="K48" s="4">
         <v>-7.69</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L48" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>99</v>
       </c>
@@ -2890,8 +3085,11 @@
       <c r="K49" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L49" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>101</v>
       </c>
@@ -2925,8 +3123,11 @@
       <c r="K50" s="5">
         <v>0.66</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L50" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>103</v>
       </c>
@@ -2960,8 +3161,11 @@
       <c r="K51" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L51" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>105</v>
       </c>
@@ -2983,20 +3187,23 @@
       <c r="G52">
         <v>0</v>
       </c>
-      <c r="H52" t="s">
-        <v>263</v>
-      </c>
-      <c r="I52" t="s">
-        <v>263</v>
-      </c>
-      <c r="J52" t="s">
-        <v>263</v>
-      </c>
-      <c r="K52" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>0</v>
+      </c>
+      <c r="J52">
+        <v>0</v>
+      </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
+      <c r="L52" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>107</v>
       </c>
@@ -3030,8 +3237,11 @@
       <c r="K53" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L53" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>109</v>
       </c>
@@ -3065,8 +3275,11 @@
       <c r="K54" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L54" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>111</v>
       </c>
@@ -3100,8 +3313,11 @@
       <c r="K55" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L55" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>113</v>
       </c>
@@ -3135,8 +3351,11 @@
       <c r="K56" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L56" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>115</v>
       </c>
@@ -3170,8 +3389,11 @@
       <c r="K57" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L57" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>117</v>
       </c>
@@ -3205,8 +3427,11 @@
       <c r="K58" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L58" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>119</v>
       </c>
@@ -3240,8 +3465,11 @@
       <c r="K59">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L59" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>121</v>
       </c>
@@ -3275,8 +3503,11 @@
       <c r="K60" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L60" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>123</v>
       </c>
@@ -3310,8 +3541,11 @@
       <c r="K61">
         <v>0.59</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L61" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>125</v>
       </c>
@@ -3345,8 +3579,11 @@
       <c r="K62" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L62" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>127</v>
       </c>
@@ -3380,8 +3617,11 @@
       <c r="K63" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L63" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>129</v>
       </c>
@@ -3415,8 +3655,11 @@
       <c r="K64">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L64" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>131</v>
       </c>
@@ -3450,8 +3693,11 @@
       <c r="K65">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L65" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>133</v>
       </c>
@@ -3473,20 +3719,23 @@
       <c r="G66">
         <v>22</v>
       </c>
-      <c r="H66">
+      <c r="H66" s="4">
         <v>-1.02</v>
       </c>
-      <c r="I66">
+      <c r="I66" s="4">
         <v>-1.17</v>
       </c>
-      <c r="J66">
+      <c r="J66" s="4">
         <v>-1.41</v>
       </c>
-      <c r="K66">
+      <c r="K66" s="4">
         <v>-1.96</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L66" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>135</v>
       </c>
@@ -3518,10 +3767,13 @@
         <v>0.47</v>
       </c>
       <c r="K67">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+        <v>0.67</v>
+      </c>
+      <c r="L67" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>137</v>
       </c>
@@ -3555,8 +3807,11 @@
       <c r="K68">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L68" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>139</v>
       </c>
@@ -3590,8 +3845,11 @@
       <c r="K69" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L69" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>141</v>
       </c>
@@ -3625,8 +3883,11 @@
       <c r="K70" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L70" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>143</v>
       </c>
@@ -3660,8 +3921,11 @@
       <c r="K71" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L71" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>145</v>
       </c>
@@ -3695,8 +3959,11 @@
       <c r="K72">
         <v>0.74</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L72" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>147</v>
       </c>
@@ -3730,8 +3997,11 @@
       <c r="K73">
         <v>0.72</v>
       </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L73" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>149</v>
       </c>
@@ -3747,12 +4017,29 @@
       <c r="E74">
         <v>0.49130000000000001</v>
       </c>
-      <c r="H74" s="3"/>
-      <c r="I74" s="3"/>
-      <c r="J74" s="3"/>
-      <c r="K74" s="3"/>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74">
+        <v>8</v>
+      </c>
+      <c r="H74" t="s">
+        <v>263</v>
+      </c>
+      <c r="I74" t="s">
+        <v>263</v>
+      </c>
+      <c r="J74" t="s">
+        <v>263</v>
+      </c>
+      <c r="K74" t="s">
+        <v>263</v>
+      </c>
+      <c r="L74" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>151</v>
       </c>
@@ -3786,8 +4073,11 @@
       <c r="K75" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L75" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>153</v>
       </c>
@@ -3821,8 +4111,11 @@
       <c r="K76" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L76" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>155</v>
       </c>
@@ -3856,8 +4149,11 @@
       <c r="K77" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L77" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>157</v>
       </c>
@@ -3891,8 +4187,11 @@
       <c r="K78" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L78" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>159</v>
       </c>
@@ -3926,8 +4225,11 @@
       <c r="K79" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L79" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>161</v>
       </c>
@@ -3961,8 +4263,11 @@
       <c r="K80" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L80" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>163</v>
       </c>
@@ -3996,8 +4301,11 @@
       <c r="K81" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L81" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>165</v>
       </c>
@@ -4031,8 +4339,11 @@
       <c r="K82" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L82" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>167</v>
       </c>
@@ -4066,8 +4377,11 @@
       <c r="K83">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L83" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>169</v>
       </c>
@@ -4101,8 +4415,11 @@
       <c r="K84">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L84" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>171</v>
       </c>
@@ -4136,8 +4453,11 @@
       <c r="K85">
         <v>0.94</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L85" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>173</v>
       </c>
@@ -4171,8 +4491,11 @@
       <c r="K86">
         <v>0.37</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L86" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>175</v>
       </c>
@@ -4206,8 +4529,11 @@
       <c r="K87" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L87" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>177</v>
       </c>
@@ -4241,8 +4567,11 @@
       <c r="K88" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L88" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>179</v>
       </c>
@@ -4276,8 +4605,11 @@
       <c r="K89" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L89" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>181</v>
       </c>
@@ -4311,8 +4643,11 @@
       <c r="K90" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L90" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>183</v>
       </c>
@@ -4346,8 +4681,11 @@
       <c r="K91" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L91" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>185</v>
       </c>
@@ -4381,8 +4719,11 @@
       <c r="K92" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L92" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>187</v>
       </c>
@@ -4416,8 +4757,11 @@
       <c r="K93" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L93" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>189</v>
       </c>
@@ -4451,8 +4795,11 @@
       <c r="K94" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L94" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>191</v>
       </c>
@@ -4486,8 +4833,11 @@
       <c r="K95">
         <v>0.48</v>
       </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L95" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>193</v>
       </c>
@@ -4518,8 +4868,11 @@
       <c r="K96" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L96" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>195</v>
       </c>
@@ -4553,8 +4906,11 @@
       <c r="K97" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L97" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>197</v>
       </c>
@@ -4588,8 +4944,11 @@
       <c r="K98" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L98" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>199</v>
       </c>
@@ -4623,8 +4982,11 @@
       <c r="K99" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L99" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>201</v>
       </c>
@@ -4658,8 +5020,11 @@
       <c r="K100" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L100" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>203</v>
       </c>
@@ -4693,8 +5058,11 @@
       <c r="K101" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L101" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>205</v>
       </c>
@@ -4728,8 +5096,11 @@
       <c r="K102">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L102" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>207</v>
       </c>
@@ -4763,8 +5134,11 @@
       <c r="K103" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L103" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>209</v>
       </c>
@@ -4798,8 +5172,11 @@
       <c r="K104" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L104" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>211</v>
       </c>
@@ -4833,8 +5210,11 @@
       <c r="K105">
         <v>0.86</v>
       </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L105" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>213</v>
       </c>
@@ -4850,12 +5230,29 @@
       <c r="E106">
         <v>0.99990000000000001</v>
       </c>
-      <c r="H106" s="3"/>
-      <c r="I106" s="3"/>
-      <c r="J106" s="3"/>
-      <c r="K106" s="3"/>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F106">
+        <v>69</v>
+      </c>
+      <c r="G106">
+        <v>31</v>
+      </c>
+      <c r="H106">
+        <v>0.59</v>
+      </c>
+      <c r="I106">
+        <v>0.7</v>
+      </c>
+      <c r="J106">
+        <v>0.87</v>
+      </c>
+      <c r="K106" t="s">
+        <v>263</v>
+      </c>
+      <c r="L106" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>215</v>
       </c>
@@ -4889,8 +5286,11 @@
       <c r="K107">
         <v>0</v>
       </c>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L107" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>217</v>
       </c>
@@ -4924,8 +5324,11 @@
       <c r="K108">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L108" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>219</v>
       </c>
@@ -4956,8 +5359,11 @@
       <c r="K109" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L109" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>221</v>
       </c>
@@ -4991,8 +5397,11 @@
       <c r="K110" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L110" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>223</v>
       </c>
@@ -5026,8 +5435,11 @@
       <c r="K111" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L111" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>225</v>
       </c>
@@ -5061,8 +5473,11 @@
       <c r="K112">
         <v>0.81</v>
       </c>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L112" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>227</v>
       </c>
@@ -5096,8 +5511,11 @@
       <c r="K113" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L113" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>229</v>
       </c>
@@ -5131,8 +5549,11 @@
       <c r="K114" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L114" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>231</v>
       </c>
@@ -5148,12 +5569,29 @@
       <c r="E115">
         <v>0.99809999999999999</v>
       </c>
-      <c r="H115" s="3"/>
-      <c r="I115" s="3"/>
-      <c r="J115" s="3"/>
-      <c r="K115" s="3"/>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F115">
+        <v>5</v>
+      </c>
+      <c r="G115">
+        <v>95</v>
+      </c>
+      <c r="H115" t="s">
+        <v>263</v>
+      </c>
+      <c r="I115" t="s">
+        <v>263</v>
+      </c>
+      <c r="J115" t="s">
+        <v>263</v>
+      </c>
+      <c r="K115" t="s">
+        <v>263</v>
+      </c>
+      <c r="L115" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>233</v>
       </c>
@@ -5187,8 +5625,11 @@
       <c r="K116" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L116" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>235</v>
       </c>
@@ -5209,7 +5650,7 @@
       <c r="J117" s="3"/>
       <c r="K117" s="3"/>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>237</v>
       </c>
@@ -5230,7 +5671,7 @@
       <c r="J118" s="3"/>
       <c r="K118" s="3"/>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>239</v>
       </c>
@@ -5264,8 +5705,11 @@
       <c r="K119" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L119" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>241</v>
       </c>
@@ -5299,8 +5743,11 @@
       <c r="K120" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L120" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>243</v>
       </c>
@@ -5334,8 +5781,11 @@
       <c r="K121" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L121" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>245</v>
       </c>
@@ -5369,8 +5819,11 @@
       <c r="K122" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L122" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>247</v>
       </c>
@@ -5404,8 +5857,11 @@
       <c r="K123" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L123" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>249</v>
       </c>
@@ -5439,8 +5895,11 @@
       <c r="K124" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L124" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>251</v>
       </c>
@@ -5474,8 +5933,11 @@
       <c r="K125">
         <v>0</v>
       </c>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L125" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>253</v>
       </c>
@@ -5509,8 +5971,11 @@
       <c r="K126" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L126" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>255</v>
       </c>
@@ -5544,8 +6009,11 @@
       <c r="K127" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L127" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>257</v>
       </c>
@@ -5578,6 +6046,9 @@
       </c>
       <c r="K128">
         <v>0.62</v>
+      </c>
+      <c r="L128" t="s">
+        <v>267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>